<commit_message>
Upload file personalia via web
</commit_message>
<xml_diff>
--- a/data/personalia/1 JAK (LAA).xlsx
+++ b/data/personalia/1 JAK (LAA).xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/047618f1b9410114/Desktop/p3ste-app/Fix/Personalia/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\OneDrive\Desktop\p3ste-app\Fix\Personalia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{2B126D94-E813-42C9-ADCA-5A3521B3FC1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C69F68E6-1F47-4DE6-AB31-6024768E660E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07F79540-3EC8-43BC-BC69-4EA818B1DBD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1985,6 +1985,9 @@
       <c r="K4" s="6">
         <v>34304</v>
       </c>
+      <c r="L4" s="6">
+        <v>46085</v>
+      </c>
       <c r="M4" s="6">
         <v>20455</v>
       </c>
@@ -7173,6 +7176,9 @@
       </c>
       <c r="K113" s="6">
         <v>40163</v>
+      </c>
+      <c r="L113" s="6">
+        <v>46085</v>
       </c>
       <c r="M113" s="6">
         <v>20455</v>

</xml_diff>